<commit_message>
Rest and Spread Operator
</commit_message>
<xml_diff>
--- a/Road Map.xlsx
+++ b/Road Map.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2081126\aem_practice\My Tectra AEM Git\My-Tectra-AEM-Tutorials-Practice\Interview Guide\React Js\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2081126\aem_practice\JS-and-React-Js\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37A28391-FBBB-49B4-9CE9-0A10C8C8ADAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64672F42-BC08-4F48-A0C9-095AF13D11AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -572,7 +572,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -591,6 +591,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -604,11 +610,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -931,13 +938,13 @@
       <c r="B2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="4" t="s">
         <v>11</v>
       </c>
       <c r="F2" s="2" t="s">
@@ -951,16 +958,16 @@
       <c r="A3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="4" t="s">
         <v>18</v>
       </c>
       <c r="F3" s="2" t="s">

</xml_diff>